<commit_message>
commmission & max loss
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$7</f>
+              <f>'Daily'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$7</f>
+              <f>'Daily'!$B$2:$B$8</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$7</f>
+              <f>'Daily'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$7</f>
+              <f>'Daily'!$C$2:$C$8</f>
             </numRef>
           </val>
         </ser>
@@ -585,6 +585,86 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>P&amp;L by Conviction Tier</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analysis'!B28</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analysis'!$A$29:$A$31</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analysis'!$B$29:$B$31</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -697,6 +777,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1011,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-06 17:52 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-07-07 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$26)</f>
+        <f>SUM(Trades!$N$2:$N$30)</f>
         <v/>
       </c>
     </row>
@@ -1033,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1044,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$26,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$30,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1055,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$26,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$30,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1066,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$26,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$26,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$30,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$30,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1077,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$26,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$26,"&gt;0")/SUMIF(Trades!$N$2:$N$26,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$30,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$30,"&gt;0")/SUMIF(Trades!$N$2:$N$30,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1088,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$7)</f>
+        <f>MAX(Daily!$B$2:$B$8)</f>
         <v/>
       </c>
     </row>
@@ -1099,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$7)</f>
+        <f>MIN(Daily!$B$2:$B$8)</f>
         <v/>
       </c>
     </row>
@@ -1115,7 +1217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1134,6 +1236,7 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1215,6 +1318,11 @@
       <c r="P1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>Conviction</t>
         </is>
       </c>
     </row>
@@ -1263,6 +1371,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -1321,6 +1430,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q3" s="10" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n">
@@ -1379,6 +1489,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -1437,6 +1548,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -1495,6 +1607,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -1553,6 +1666,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
@@ -1611,6 +1725,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n">
@@ -1669,6 +1784,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
@@ -1711,6 +1827,7 @@
           <t>Orphaned/manual</t>
         </is>
       </c>
+      <c r="Q10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -1771,6 +1888,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -1831,6 +1949,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -1891,6 +2010,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
@@ -1951,6 +2071,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -2011,6 +2132,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
@@ -2053,6 +2175,7 @@
           <t>Orphaned/manual</t>
         </is>
       </c>
+      <c r="Q16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
@@ -2095,6 +2218,7 @@
           <t>Orphaned/manual</t>
         </is>
       </c>
+      <c r="Q17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -2155,6 +2279,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -2215,6 +2340,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -2273,6 +2399,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -2331,6 +2458,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
@@ -2389,6 +2517,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
@@ -2451,6 +2580,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q23" s="10" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
@@ -2513,6 +2643,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q24" s="10" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -2575,6 +2706,7 @@
           <t>Closed</t>
         </is>
       </c>
+      <c r="Q25" s="10" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
@@ -2635,6 +2767,275 @@
       <c r="P26" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q26" s="10" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>07-07 10:19</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>07-07 10:48</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>0.377143</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>0.4500000000000002</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>45.64</v>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>0.4848</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>0.1932</v>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P27" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q27" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 3/5 | ADX✓ slope✗ agree✓(QQQ+IWM) early✓ tape✗(6x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>07-07 10:20</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>07-07 10:37</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" s="10" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="I28" s="10" t="n">
+        <v>0.5299999999999998</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>36.28</v>
+      </c>
+      <c r="K28" s="10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>0.5769</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>Trail (new)</t>
+        </is>
+      </c>
+      <c r="P28" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q28" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 3/5 | ADX✓ slope✗ agree✓(SPY+IWM) early✓ tape✗(8x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>07-07 10:44</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>07-07 10:47</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H29" s="10" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I29" s="10" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>26.31</v>
+      </c>
+      <c r="K29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>-0.3222</v>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>-87</v>
+      </c>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P29" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q29" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 2/5 | ADX✗ slope✗ agree✓(QQQ) early✓ tape✗(8x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>07-07 12:09</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>07-07 12:14</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H30" s="10" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I30" s="10" t="n">
+        <v>0.2299999999999999</v>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>35.34</v>
+      </c>
+      <c r="K30" s="10" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>-0.3429</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>-48</v>
+      </c>
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P30" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q30" s="10" t="inlineStr">
+        <is>
+          <t>LOW 0/5 | ADX✓ slope✓ agree✗ early✗ tape✗(22x) inv−2</t>
         </is>
       </c>
     </row>
@@ -2649,7 +3050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2699,7 +3100,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$26)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$30)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -2707,11 +3108,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$26="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$30="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$26&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$30&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -2726,7 +3127,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$26)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$30)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -2734,11 +3135,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$26="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$30="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$26&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$30&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -2753,7 +3154,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$26)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$30)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -2761,11 +3162,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$26="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$30="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$26&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$30&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -2780,7 +3181,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$26)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$30)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -2788,11 +3189,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$26="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$30="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$26&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$30&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -2807,7 +3208,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$26)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$30)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -2815,11 +3216,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$26="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$30="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$26&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$30&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -2834,7 +3235,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$26)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$30)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -2842,15 +3243,42 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$26="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$30="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$26,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$26&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$30&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
         <f>D7-E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07/07</t>
+        </is>
+      </c>
+      <c r="B8" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$30)</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>SUM($B$2:B8)</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>D8-E8</f>
         <v/>
       </c>
     </row>
@@ -2865,7 +3293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2910,15 +3338,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$B$2:$B$26,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$B$2:$B$30,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$26,A3,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$30,A3,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$26,A3,Trades!$N$2:$N$26,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$30,A3,Trades!$N$2:$N$30,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -2929,15 +3357,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$B$2:$B$26,A4)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$B$2:$B$30,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS(Trades!$B$2:$B$26,A4,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$30,A4,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$26,A4,Trades!$N$2:$N$26,"&gt;0")/C4)</f>
+        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$30,A4,Trades!$N$2:$N$30,"&gt;0")/C4)</f>
         <v/>
       </c>
     </row>
@@ -2948,15 +3376,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$B$2:$B$26,A5)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$B$2:$B$30,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS(Trades!$B$2:$B$26,A5,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$30,A5,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$26,A5,Trades!$N$2:$N$26,"&gt;0")/C5)</f>
+        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$30,A5,Trades!$N$2:$N$30,"&gt;0")/C5)</f>
         <v/>
       </c>
     </row>
@@ -2996,11 +3424,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$O$2:$O$26,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$26,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$30,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -3015,11 +3443,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$O$2:$O$26,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$26,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$30,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -3034,11 +3462,11 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$O$2:$O$26,A12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIF(Trades!$O$2:$O$26,A12)</f>
+        <f>COUNTIF(Trades!$O$2:$O$30,A12)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -3053,11 +3481,11 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$O$2:$O$26,A13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIF(Trades!$O$2:$O$26,A13)</f>
+        <f>COUNTIF(Trades!$O$2:$O$30,A13)</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -3096,11 +3524,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,9)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$26,9,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,9,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3111,11 +3539,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,10)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$26,10,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,10,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3126,11 +3554,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,11)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$26,11,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,11,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3141,11 +3569,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,12)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$26,12,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,12,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3156,11 +3584,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,13)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$26,13,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,13,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3171,11 +3599,11 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,14)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Trades!$G$2:$G$26,14,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,14,Trades!$P$2:$P$30,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3186,11 +3614,97 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$26,Trades!$G$2:$G$26,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,15)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Trades!$G$2:$G$26,15,Trades!$P$2:$P$26,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$30,15,Trades!$P$2:$P$30,"Closed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>By Conviction Tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>P&amp;L $</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Trades</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Win rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B29" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$Q$2:$Q$30,A29&amp;" *")</f>
+        <v/>
+      </c>
+      <c r="C29">
+        <f>COUNTIFS(Trades!$Q$2:$Q$30,A29&amp;" *",Trades!$P$2:$P$30,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D29" s="13">
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$30,A29&amp;" *",Trades!$N$2:$N$30,"&gt;0")/C29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$Q$2:$Q$30,A30&amp;" *")</f>
+        <v/>
+      </c>
+      <c r="C30">
+        <f>COUNTIFS(Trades!$Q$2:$Q$30,A30&amp;" *",Trades!$P$2:$P$30,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D30" s="13">
+        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$30,A30&amp;" *",Trades!$N$2:$N$30,"&gt;0")/C30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B31" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$Q$2:$Q$30,A31&amp;" *")</f>
+        <v/>
+      </c>
+      <c r="C31">
+        <f>COUNTIFS(Trades!$Q$2:$Q$30,A31&amp;" *",Trades!$P$2:$P$30,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D31" s="13">
+        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$30,A31&amp;" *",Trades!$N$2:$N$30,"&gt;0")/C31)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
conviction score based entry and exits
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$8</f>
+              <f>'Daily'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$8</f>
+              <f>'Daily'!$B$2:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$8</f>
+              <f>'Daily'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$8</f>
+              <f>'Daily'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-07 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-07-08 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$30)</f>
+        <f>SUM(Trades!$N$2:$N$37)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$30,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$37,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$30,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$37,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$30,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$30,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$37,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$37,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$30,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$30,"&gt;0")/SUMIF(Trades!$N$2:$N$30,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$37,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$37,"&gt;0")/SUMIF(Trades!$N$2:$N$37,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$8)</f>
+        <f>MAX(Daily!$B$2:$B$9)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,29 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$8)</f>
+        <f>MIN(Daily!$B$2:$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Commissions $</t>
+        </is>
+      </c>
+      <c r="B12" s="4">
+        <f>SUM(Trades!$R$2:$R$37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Net after fees $</t>
+        </is>
+      </c>
+      <c r="B13" s="4">
+        <f>B4-B12</f>
         <v/>
       </c>
     </row>
@@ -1217,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1237,6 +1259,7 @@
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1323,6 +1346,11 @@
       <c r="Q1" s="8" t="inlineStr">
         <is>
           <t>Conviction</t>
+        </is>
+      </c>
+      <c r="R1" s="8" t="inlineStr">
+        <is>
+          <t>Commission</t>
         </is>
       </c>
     </row>
@@ -1372,6 +1400,7 @@
         </is>
       </c>
       <c r="Q2" s="10" t="inlineStr"/>
+      <c r="R2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -1431,6 +1460,7 @@
         </is>
       </c>
       <c r="Q3" s="10" t="inlineStr"/>
+      <c r="R3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n">
@@ -1490,6 +1520,7 @@
         </is>
       </c>
       <c r="Q4" s="10" t="inlineStr"/>
+      <c r="R4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -1549,6 +1580,7 @@
         </is>
       </c>
       <c r="Q5" s="10" t="inlineStr"/>
+      <c r="R5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -1608,6 +1640,7 @@
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr"/>
+      <c r="R6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -1667,6 +1700,7 @@
         </is>
       </c>
       <c r="Q7" s="10" t="inlineStr"/>
+      <c r="R7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
@@ -1726,6 +1760,7 @@
         </is>
       </c>
       <c r="Q8" s="10" t="inlineStr"/>
+      <c r="R8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n">
@@ -1785,6 +1820,7 @@
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr"/>
+      <c r="R9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
@@ -1828,6 +1864,7 @@
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr"/>
+      <c r="R10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -1889,6 +1926,7 @@
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr"/>
+      <c r="R11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -1950,6 +1988,7 @@
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr"/>
+      <c r="R12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -2011,6 +2050,7 @@
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr"/>
+      <c r="R13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
@@ -2072,6 +2112,7 @@
         </is>
       </c>
       <c r="Q14" s="10" t="inlineStr"/>
+      <c r="R14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -2133,6 +2174,7 @@
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr"/>
+      <c r="R15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
@@ -2176,6 +2218,7 @@
         </is>
       </c>
       <c r="Q16" s="10" t="inlineStr"/>
+      <c r="R16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
@@ -2219,6 +2262,7 @@
         </is>
       </c>
       <c r="Q17" s="10" t="inlineStr"/>
+      <c r="R17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -2280,6 +2324,7 @@
         </is>
       </c>
       <c r="Q18" s="10" t="inlineStr"/>
+      <c r="R18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -2341,6 +2386,7 @@
         </is>
       </c>
       <c r="Q19" s="10" t="inlineStr"/>
+      <c r="R19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -2400,6 +2446,7 @@
         </is>
       </c>
       <c r="Q20" s="10" t="inlineStr"/>
+      <c r="R20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -2459,6 +2506,7 @@
         </is>
       </c>
       <c r="Q21" s="10" t="inlineStr"/>
+      <c r="R21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
@@ -2518,6 +2566,7 @@
         </is>
       </c>
       <c r="Q22" s="10" t="inlineStr"/>
+      <c r="R22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
@@ -2581,6 +2630,7 @@
         </is>
       </c>
       <c r="Q23" s="10" t="inlineStr"/>
+      <c r="R23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
@@ -2644,6 +2694,7 @@
         </is>
       </c>
       <c r="Q24" s="10" t="inlineStr"/>
+      <c r="R24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -2707,6 +2758,7 @@
         </is>
       </c>
       <c r="Q25" s="10" t="inlineStr"/>
+      <c r="R25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
@@ -2770,6 +2822,7 @@
         </is>
       </c>
       <c r="Q26" s="10" t="inlineStr"/>
+      <c r="R26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
@@ -2837,6 +2890,7 @@
           <t>MEDIUM 3/5 | ADX✓ slope✗ agree✓(QQQ+IWM) early✓ tape✗(6x)</t>
         </is>
       </c>
+      <c r="R27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
@@ -2904,6 +2958,7 @@
           <t>MEDIUM 3/5 | ADX✓ slope✗ agree✓(SPY+IWM) early✓ tape✗(8x)</t>
         </is>
       </c>
+      <c r="R28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -2971,6 +3026,7 @@
           <t>MEDIUM 2/5 | ADX✗ slope✗ agree✓(QQQ) early✓ tape✗(8x)</t>
         </is>
       </c>
+      <c r="R29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
@@ -3037,6 +3093,497 @@
         <is>
           <t>LOW 0/5 | ADX✓ slope✓ agree✗ early✗ tape✗(22x) inv−2</t>
         </is>
+      </c>
+      <c r="R30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>07-08 10:44</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>07-08 10:54</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H31" s="10" t="n">
+        <v>0.407143</v>
+      </c>
+      <c r="I31" s="10" t="n">
+        <v>0.425714</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>25.91</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>0.2035</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>0.04559999999999999</v>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O31" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P31" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q31" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 3/5 | ADX✗ slope✓ agree✓(SPY+QQQ) early✓ tape✗(12x)</t>
+        </is>
+      </c>
+      <c r="R31" s="4" t="n">
+        <v>13.87</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>07-08 10:52</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>07-08 10:55</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H32" s="10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I32" s="10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>25.03</v>
+      </c>
+      <c r="K32" s="10" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>-70</v>
+      </c>
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P32" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q32" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 3/5 | ADX✗ slope✓ agree✓(QQQ) early✓ tape✗(12x)</t>
+        </is>
+      </c>
+      <c r="R32" s="4" t="n">
+        <v>12.46</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>07-08 11:19</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>07-08 11:36</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H33" s="10" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="I33" s="10" t="n">
+        <v>0.483333</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="L33" s="6" t="n">
+        <v>0.2558</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O33" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P33" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q33" s="10" t="inlineStr">
+        <is>
+          <t>LOW -1/5 | ADX✗ slope✗ agree✓(SPY+QQQ) early✗ tape✗(18x) inv−2</t>
+        </is>
+      </c>
+      <c r="R33" s="4" t="n">
+        <v>6.32</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>07-08 11:29</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>07-08 11:38</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H34" s="10" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="I34" s="10" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>25.17</v>
+      </c>
+      <c r="K34" s="10" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>-0.2826</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>-39</v>
+      </c>
+      <c r="O34" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P34" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q34" s="10" t="inlineStr">
+        <is>
+          <t>LOW 0/5 | ADX✗ slope✓ agree✓(SPY) early✗ tape✗(16x) inv−2</t>
+        </is>
+      </c>
+      <c r="R34" s="4" t="n">
+        <v>5.41</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>07-08 11:31</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>07-08 11:39</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H35" s="10" t="n">
+        <v>0.453333</v>
+      </c>
+      <c r="I35" s="10" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="K35" s="10" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="L35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="6" t="n">
+        <v>-0.3162</v>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>-43</v>
+      </c>
+      <c r="O35" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P35" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q35" s="10" t="inlineStr">
+        <is>
+          <t>LOW -1/5 | ADX✗ slope✓ agree✗ early✗ tape✗(20x) inv−2</t>
+        </is>
+      </c>
+      <c r="R35" s="4" t="n">
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>07-08 13:31</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>07-08 13:39</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H36" s="10" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I36" s="10" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J36" s="10" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="K36" s="10" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>0.0244</v>
+      </c>
+      <c r="M36" s="6" t="n">
+        <v>-0.1707</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>-21</v>
+      </c>
+      <c r="O36" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P36" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q36" s="10" t="inlineStr">
+        <is>
+          <t>LOW -2/5 | ADX✓ slope✓ agree✓(QQQ+IWM) early✗ tape✗(33x) inv−5</t>
+        </is>
+      </c>
+      <c r="R36" s="4" t="n">
+        <v>6.43</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>07-08 13:39</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>07-08 13:41</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H37" s="10" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I37" s="10" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="J37" s="10" t="n">
+        <v>33.38</v>
+      </c>
+      <c r="K37" s="10" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="L37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="6" t="n">
+        <v>-0.09759999999999999</v>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>-12</v>
+      </c>
+      <c r="O37" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P37" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q37" s="10" t="inlineStr">
+        <is>
+          <t>LOW -2/5 | ADX✓ slope✓ agree✓(SPY+IWM) early✗ tape✗(25x) inv−5</t>
+        </is>
+      </c>
+      <c r="R37" s="4" t="n">
+        <v>4.98</v>
       </c>
     </row>
   </sheetData>
@@ -3050,7 +3597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3100,7 +3647,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -3108,11 +3655,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -3127,7 +3674,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -3135,11 +3682,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -3154,7 +3701,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3162,11 +3709,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -3181,7 +3728,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3189,11 +3736,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -3208,7 +3755,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3216,11 +3763,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -3235,7 +3782,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -3243,11 +3790,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -3262,7 +3809,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$30)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$37)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -3270,15 +3817,42 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$30="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$37="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$30,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$30&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$37&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
         <f>D8-E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07/08</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$37)</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>SUM($B$2:B9)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>D9-E9</f>
         <v/>
       </c>
     </row>
@@ -3338,15 +3912,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$B$2:$B$30,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$B$2:$B$37,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$30,A3,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$37,A3,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$30,A3,Trades!$N$2:$N$30,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$37,A3,Trades!$N$2:$N$37,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -3357,15 +3931,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$B$2:$B$30,A4)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$B$2:$B$37,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS(Trades!$B$2:$B$30,A4,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$37,A4,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$30,A4,Trades!$N$2:$N$30,"&gt;0")/C4)</f>
+        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$37,A4,Trades!$N$2:$N$37,"&gt;0")/C4)</f>
         <v/>
       </c>
     </row>
@@ -3376,15 +3950,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$B$2:$B$30,A5)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$B$2:$B$37,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS(Trades!$B$2:$B$30,A5,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$37,A5,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$30,A5,Trades!$N$2:$N$30,"&gt;0")/C5)</f>
+        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$37,A5,Trades!$N$2:$N$37,"&gt;0")/C5)</f>
         <v/>
       </c>
     </row>
@@ -3424,11 +3998,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$30,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$37,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -3443,11 +4017,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$30,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$37,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -3462,11 +4036,11 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIF(Trades!$O$2:$O$30,A12)</f>
+        <f>COUNTIF(Trades!$O$2:$O$37,A12)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -3481,11 +4055,11 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$O$2:$O$30,A13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIF(Trades!$O$2:$O$30,A13)</f>
+        <f>COUNTIF(Trades!$O$2:$O$37,A13)</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -3524,11 +4098,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,9)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$30,9,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,9,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3539,11 +4113,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,10)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$30,10,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,10,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3554,11 +4128,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,11)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$30,11,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,11,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3569,11 +4143,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,12)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$30,12,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,12,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3584,11 +4158,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,13)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$30,13,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,13,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3599,11 +4173,11 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,14)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Trades!$G$2:$G$30,14,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,14,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3614,11 +4188,11 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$G$2:$G$30,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,15)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Trades!$G$2:$G$30,15,Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$37,15,Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -3658,15 +4232,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$Q$2:$Q$30,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$Q$2:$Q$37,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$30,A29&amp;" *",Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$37,A29&amp;" *",Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$30,A29&amp;" *",Trades!$N$2:$N$30,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$37,A29&amp;" *",Trades!$N$2:$N$37,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>
@@ -3677,15 +4251,15 @@
         </is>
       </c>
       <c r="B30" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$Q$2:$Q$30,A30&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$Q$2:$Q$37,A30&amp;" *")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Trades!$Q$2:$Q$30,A30&amp;" *",Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$37,A30&amp;" *",Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
       <c r="D30" s="13">
-        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$30,A30&amp;" *",Trades!$N$2:$N$30,"&gt;0")/C30)</f>
+        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$37,A30&amp;" *",Trades!$N$2:$N$37,"&gt;0")/C30)</f>
         <v/>
       </c>
     </row>
@@ -3696,15 +4270,15 @@
         </is>
       </c>
       <c r="B31" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$30,Trades!$Q$2:$Q$30,A31&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$Q$2:$Q$37,A31&amp;" *")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS(Trades!$Q$2:$Q$30,A31&amp;" *",Trades!$P$2:$P$30,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$37,A31&amp;" *",Trades!$P$2:$P$37,"Closed")</f>
         <v/>
       </c>
       <c r="D31" s="13">
-        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$30,A31&amp;" *",Trades!$N$2:$N$30,"&gt;0")/C31)</f>
+        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$37,A31&amp;" *",Trades!$N$2:$N$37,"&gt;0")/C31)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
logic to fix orphaned trades
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$9</f>
+              <f>'Daily'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$9</f>
+              <f>'Daily'!$B$2:$B$10</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$9</f>
+              <f>'Daily'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$9</f>
+              <f>'Daily'!$C$2:$C$10</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-08 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-07-09 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$37)</f>
+        <f>SUM(Trades!$N$2:$N$43)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$37,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$43,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$37,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$43,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$37,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$37,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$43,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$43,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$37,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$37,"&gt;0")/SUMIF(Trades!$N$2:$N$37,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$43,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$43,"&gt;0")/SUMIF(Trades!$N$2:$N$43,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$9)</f>
+        <f>MAX(Daily!$B$2:$B$10)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$9)</f>
+        <f>MIN(Daily!$B$2:$B$10)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$37)</f>
+        <f>SUM(Trades!$R$2:$R$43)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R37"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3586,6 +3586,360 @@
         <v>4.98</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>07-09 10:26</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>07-09 10:27</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H38" s="10" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I38" s="10" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J38" s="10" t="n">
+        <v>43.15</v>
+      </c>
+      <c r="K38" s="10" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="L38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="6" t="n">
+        <v>-0.1212</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>-52</v>
+      </c>
+      <c r="O38" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P38" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q38" s="10" t="inlineStr">
+        <is>
+          <t>HIGH 5/5 | ADX✓ slope✓ agree✓(SPY+IWM) early✓ tape✓(4x)</t>
+        </is>
+      </c>
+      <c r="R38" s="4" t="n">
+        <v>30.14</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>CONDOR</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>07-09 11:05</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>07-09 13:11</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>126</v>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H39" s="10" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="I39" s="10" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>11.94</v>
+      </c>
+      <c r="K39" s="10" t="n"/>
+      <c r="L39" s="6" t="n">
+        <v>0.2432</v>
+      </c>
+      <c r="M39" s="6" t="n">
+        <v>-0.6486</v>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>-96</v>
+      </c>
+      <c r="O39" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P39" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q39" s="10" t="inlineStr"/>
+      <c r="R39" s="4" t="n">
+        <v>10.78</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>CONDOR</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>07-09 11:07</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>07-09 11:43</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H40" s="10" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="I40" s="10" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J40" s="10" t="n">
+        <v>14.48</v>
+      </c>
+      <c r="K40" s="10" t="n"/>
+      <c r="L40" s="6" t="n">
+        <v>0.08019999999999999</v>
+      </c>
+      <c r="M40" s="6" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>-53</v>
+      </c>
+      <c r="O40" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P40" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q40" s="10" t="inlineStr"/>
+      <c r="R40" s="4" t="n">
+        <v>19.76</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>CONDOR</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>07-09 11:08</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H41" s="10" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I41" s="10" t="n"/>
+      <c r="J41" s="10" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="K41" s="10" t="n"/>
+      <c r="L41" s="6" t="n"/>
+      <c r="M41" s="6" t="n"/>
+      <c r="N41" s="4" t="n"/>
+      <c r="O41" s="10" t="inlineStr"/>
+      <c r="P41" s="10" t="inlineStr">
+        <is>
+          <t>Orphaned/manual</t>
+        </is>
+      </c>
+      <c r="Q41" s="10" t="inlineStr"/>
+      <c r="R41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>CONDOR</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>07-09 11:42</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>07-09 13:11</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="n">
+        <v>89</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H42" s="10" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="I42" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J42" s="10" t="n">
+        <v>18.96</v>
+      </c>
+      <c r="K42" s="10" t="n"/>
+      <c r="L42" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M42" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="O42" s="10" t="inlineStr">
+        <is>
+          <t>Trail (new)</t>
+        </is>
+      </c>
+      <c r="P42" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q42" s="10" t="inlineStr"/>
+      <c r="R42" s="4" t="n">
+        <v>5.21</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>07-09 11:46</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H43" s="10" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I43" s="10" t="n"/>
+      <c r="J43" s="10" t="n">
+        <v>34.27</v>
+      </c>
+      <c r="K43" s="10" t="n"/>
+      <c r="L43" s="6" t="n"/>
+      <c r="M43" s="6" t="n"/>
+      <c r="N43" s="4" t="n"/>
+      <c r="O43" s="10" t="inlineStr"/>
+      <c r="P43" s="10" t="inlineStr">
+        <is>
+          <t>Orphaned/manual</t>
+        </is>
+      </c>
+      <c r="Q43" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 2/5 | ADX✓ slope✓ agree✓(IWM) early✗ tape✗(13x) inv−1</t>
+        </is>
+      </c>
+      <c r="R43" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3597,7 +3951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3647,7 +4001,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -3655,11 +4009,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -3674,7 +4028,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -3682,11 +4036,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -3701,7 +4055,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3709,11 +4063,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -3728,7 +4082,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3736,11 +4090,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -3755,7 +4109,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3763,11 +4117,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -3782,7 +4136,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -3790,11 +4144,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -3809,7 +4163,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -3817,11 +4171,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -3836,7 +4190,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$37)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$43)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -3844,15 +4198,42 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$37="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$43="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$37,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$37&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$43&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
         <f>D9-E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07/09</t>
+        </is>
+      </c>
+      <c r="B10" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$43)</f>
+        <v/>
+      </c>
+      <c r="C10" s="11">
+        <f>SUM($B$2:B10)</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$43="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$43,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$43&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>D10-E10</f>
         <v/>
       </c>
     </row>
@@ -3912,15 +4293,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$B$2:$B$37,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$B$2:$B$43,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$37,A3,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$43,A3,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$37,A3,Trades!$N$2:$N$37,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$43,A3,Trades!$N$2:$N$43,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -3931,15 +4312,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$B$2:$B$37,A4)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$B$2:$B$43,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS(Trades!$B$2:$B$37,A4,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$43,A4,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$37,A4,Trades!$N$2:$N$37,"&gt;0")/C4)</f>
+        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$43,A4,Trades!$N$2:$N$43,"&gt;0")/C4)</f>
         <v/>
       </c>
     </row>
@@ -3950,15 +4331,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$B$2:$B$37,A5)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$B$2:$B$43,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS(Trades!$B$2:$B$37,A5,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$43,A5,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$37,A5,Trades!$N$2:$N$37,"&gt;0")/C5)</f>
+        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$43,A5,Trades!$N$2:$N$43,"&gt;0")/C5)</f>
         <v/>
       </c>
     </row>
@@ -3998,11 +4379,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$O$2:$O$43,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$37,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$43,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -4017,11 +4398,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$O$2:$O$43,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$37,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$43,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -4036,11 +4417,11 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$O$2:$O$43,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIF(Trades!$O$2:$O$37,A12)</f>
+        <f>COUNTIF(Trades!$O$2:$O$43,A12)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -4055,11 +4436,11 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$O$2:$O$37,A13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$O$2:$O$43,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIF(Trades!$O$2:$O$37,A13)</f>
+        <f>COUNTIF(Trades!$O$2:$O$43,A13)</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -4098,11 +4479,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,9)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$37,9,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,9,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4113,11 +4494,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,10)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$37,10,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,10,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4128,11 +4509,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,11)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$37,11,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,11,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4143,11 +4524,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,12)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$37,12,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,12,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4158,11 +4539,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,13)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$37,13,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,13,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4173,11 +4554,11 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,14)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Trades!$G$2:$G$37,14,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,14,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4188,11 +4569,11 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$G$2:$G$37,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$G$2:$G$43,15)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Trades!$G$2:$G$37,15,Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$43,15,Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -4232,15 +4613,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$Q$2:$Q$37,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$Q$2:$Q$43,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$37,A29&amp;" *",Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$43,A29&amp;" *",Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$37,A29&amp;" *",Trades!$N$2:$N$37,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$43,A29&amp;" *",Trades!$N$2:$N$43,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>
@@ -4251,15 +4632,15 @@
         </is>
       </c>
       <c r="B30" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$Q$2:$Q$37,A30&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$Q$2:$Q$43,A30&amp;" *")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Trades!$Q$2:$Q$37,A30&amp;" *",Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$43,A30&amp;" *",Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
       <c r="D30" s="13">
-        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$37,A30&amp;" *",Trades!$N$2:$N$37,"&gt;0")/C30)</f>
+        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$43,A30&amp;" *",Trades!$N$2:$N$43,"&gt;0")/C30)</f>
         <v/>
       </c>
     </row>
@@ -4270,15 +4651,15 @@
         </is>
       </c>
       <c r="B31" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$37,Trades!$Q$2:$Q$37,A31&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$43,Trades!$Q$2:$Q$43,A31&amp;" *")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS(Trades!$Q$2:$Q$37,A31&amp;" *",Trades!$P$2:$P$37,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$43,A31&amp;" *",Trades!$P$2:$P$43,"Closed")</f>
         <v/>
       </c>
       <c r="D31" s="13">
-        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$37,A31&amp;" *",Trades!$N$2:$N$37,"&gt;0")/C31)</f>
+        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$43,A31&amp;" *",Trades!$N$2:$N$43,"&gt;0")/C31)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
code fixes & XSP migration
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$11</f>
+              <f>'Daily'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$11</f>
+              <f>'Daily'!$B$2:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$11</f>
+              <f>'Daily'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$11</f>
+              <f>'Daily'!$C$2:$C$13</f>
             </numRef>
           </val>
         </ser>
@@ -383,12 +383,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analysis'!$A$3:$A$5</f>
+              <f>'Analysis'!$A$3:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analysis'!$B$3:$B$5</f>
+              <f>'Analysis'!$B$3:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -453,7 +453,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analysis'!B9</f>
+              <f>'Analysis'!B10</f>
             </strRef>
           </tx>
           <spPr>
@@ -463,12 +463,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analysis'!$A$10:$A$13</f>
+              <f>'Analysis'!$A$11:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analysis'!$B$10:$B$13</f>
+              <f>'Analysis'!$B$11:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -533,7 +533,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analysis'!B17</f>
+              <f>'Analysis'!B18</f>
             </strRef>
           </tx>
           <spPr>
@@ -543,12 +543,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analysis'!$A$18:$A$24</f>
+              <f>'Analysis'!$A$19:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analysis'!$B$18:$B$24</f>
+              <f>'Analysis'!$B$19:$B$25</f>
             </numRef>
           </val>
         </ser>
@@ -613,7 +613,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analysis'!B28</f>
+              <f>'Analysis'!B29</f>
             </strRef>
           </tx>
           <spPr>
@@ -623,12 +623,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analysis'!$A$29:$A$31</f>
+              <f>'Analysis'!$A$30:$A$32</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analysis'!$B$29:$B$31</f>
+              <f>'Analysis'!$B$30:$B$32</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-10 16:50 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-07-14 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$47)</f>
+        <f>SUM(Trades!$N$2:$N$50)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$47,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$50,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$47,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$50,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$47,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$47,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$50,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$50,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$47,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$47,"&gt;0")/SUMIF(Trades!$N$2:$N$47,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$50,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$50,"&gt;0")/SUMIF(Trades!$N$2:$N$50,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$11)</f>
+        <f>MAX(Daily!$B$2:$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$11)</f>
+        <f>MIN(Daily!$B$2:$B$13)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$47)</f>
+        <f>SUM(Trades!$R$2:$R$50)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R47"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4208,6 +4208,216 @@
         <v>11.37</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="9" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>07-13 10:19</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="inlineStr">
+        <is>
+          <t>07-13 10:25</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G48" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H48" s="10" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="I48" s="10" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J48" s="10" t="n">
+        <v>29.76</v>
+      </c>
+      <c r="K48" s="10" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="L48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="6" t="n">
+        <v>-0.3333</v>
+      </c>
+      <c r="N48" s="4" t="n">
+        <v>-91</v>
+      </c>
+      <c r="O48" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P48" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q48" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 3/5 | ADX✗ slope✓ agree✓(SPY+QQQ) early✓ tape✗(6x)</t>
+        </is>
+      </c>
+      <c r="R48" s="4" t="n">
+        <v>15.97</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>07-13 12:02</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>07-13 12:13</t>
+        </is>
+      </c>
+      <c r="F49" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="G49" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H49" s="10" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I49" s="10" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J49" s="10" t="n">
+        <v>34.1</v>
+      </c>
+      <c r="K49" s="10" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="L49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="6" t="n">
+        <v>-0.2222</v>
+      </c>
+      <c r="N49" s="4" t="n">
+        <v>-64</v>
+      </c>
+      <c r="O49" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P49" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q49" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 2/5 | ADX✓ slope✓ agree✓(QQQ+IWM) early✗ tape✗(26x) inv−1</t>
+        </is>
+      </c>
+      <c r="R49" s="4" t="n">
+        <v>20.39</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>XSP</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>07-14 11:07</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>07-14 11:21</t>
+        </is>
+      </c>
+      <c r="F50" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="G50" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="H50" s="10" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I50" s="10" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J50" s="10" t="n">
+        <v>33.87</v>
+      </c>
+      <c r="K50" s="10" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="L50" s="6" t="n">
+        <v>0.1633</v>
+      </c>
+      <c r="M50" s="6" t="n">
+        <v>-0.1429</v>
+      </c>
+      <c r="N50" s="4" t="n">
+        <v>-42</v>
+      </c>
+      <c r="O50" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P50" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q50" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 2/5 | ADX✓ slope✓ agree✗ early✗ tape✗(17x)</t>
+        </is>
+      </c>
+      <c r="R50" s="4" t="n">
+        <v>20.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4219,7 +4429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4269,7 +4479,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -4277,11 +4487,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -4296,7 +4506,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -4304,11 +4514,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -4323,7 +4533,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -4331,11 +4541,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -4350,7 +4560,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -4358,11 +4568,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -4377,7 +4587,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -4385,11 +4595,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -4404,7 +4614,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -4412,11 +4622,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -4431,7 +4641,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -4439,11 +4649,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -4458,7 +4668,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -4466,11 +4676,11 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
@@ -4485,7 +4695,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -4493,11 +4703,11 @@
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F10">
@@ -4512,7 +4722,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-10")*Trades!$N$2:$N$47)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-10")*Trades!$N$2:$N$50)</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -4520,15 +4730,69 @@
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-10")*(Trades!$P$2:$P$47="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-10")*(Trades!$P$2:$P$50="Closed")*1)</f>
         <v/>
       </c>
       <c r="E11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$47,"yyyy-mm-dd")="2026-07-10")*(Trades!$N$2:$N$47&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-10")*(Trades!$N$2:$N$50&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F11">
         <f>D11-E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07/13</t>
+        </is>
+      </c>
+      <c r="B12" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-13")*Trades!$N$2:$N$50)</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>SUM($B$2:B12)</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-13")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-13")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>D12-E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07/14</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-14")*Trades!$N$2:$N$50)</f>
+        <v/>
+      </c>
+      <c r="C13" s="11">
+        <f>SUM($B$2:B13)</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-14")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-14")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>D13-E13</f>
         <v/>
       </c>
     </row>
@@ -4543,7 +4807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4588,15 +4852,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$B$2:$B$47,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$47,A3,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$50,A3,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$47,A3,Trades!$N$2:$N$47,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$50,A3,Trades!$N$2:$N$50,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -4607,15 +4871,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$B$2:$B$47,A4)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS(Trades!$B$2:$B$47,A4,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$50,A4,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$47,A4,Trades!$N$2:$N$47,"&gt;0")/C4)</f>
+        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$50,A4,Trades!$N$2:$N$50,"&gt;0")/C4)</f>
         <v/>
       </c>
     </row>
@@ -4626,78 +4890,78 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$B$2:$B$47,A5)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS(Trades!$B$2:$B$47,A5,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$50,A5,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$47,A5,Trades!$N$2:$N$47,"&gt;0")/C5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$50,A5,Trades!$N$2:$N$50,"&gt;0")/C5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>XSP</t>
+        </is>
+      </c>
+      <c r="B6" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A6)</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>COUNTIFS(Trades!$B$2:$B$50,A6,Trades!$P$2:$P$50,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D6" s="13">
+        <f>IF(C6=0,0,COUNTIFS(Trades!$B$2:$B$50,A6,Trades!$N$2:$N$50,"&gt;0")/C6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>By Exit Rule</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Exit Rule</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>P&amp;L $</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Avg P&amp;L $</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Invalidation</t>
-        </is>
-      </c>
-      <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$O$2:$O$47,A10)</f>
-        <v/>
-      </c>
-      <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$47,A10)</f>
-        <v/>
-      </c>
-      <c r="D10" s="11">
-        <f>IF(C10=0,0,B10/C10)</f>
-        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hard Stop</t>
+          <t>Invalidation</t>
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$O$2:$O$47,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$47,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$50,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -4708,15 +4972,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trail (new)</t>
+          <t>Hard Stop</t>
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$O$2:$O$47,A12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIF(Trades!$O$2:$O$47,A12)</f>
+        <f>COUNTIF(Trades!$O$2:$O$50,A12)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -4727,15 +4991,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Old rule (removed)</t>
+          <t>Trail (new)</t>
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$O$2:$O$47,A13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIF(Trades!$O$2:$O$47,A13)</f>
+        <f>COUNTIF(Trades!$O$2:$O$50,A13)</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -4743,218 +5007,237 @@
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Old rule (removed)</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A14)</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>COUNTIF(Trades!$O$2:$O$50,A14)</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>IF(C14=0,0,B14/C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>By Entry Hour (ET)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Hour</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>P&amp;L $</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>9:00</t>
-        </is>
-      </c>
-      <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,9)</f>
-        <v/>
-      </c>
-      <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$47,9,Trades!$P$2:$P$47,"Closed")</f>
-        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>9:00</t>
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,9)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$47,10,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$50,9,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,10)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$47,11,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$50,10,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,11)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$47,12,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$50,11,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,12)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$47,13,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$50,12,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B23" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,13)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Trades!$G$2:$G$47,14,Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$50,13,Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,14)</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>COUNTIFS(Trades!$G$2:$G$50,14,Trades!$P$2:$P$50,"Closed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="B24" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$G$2:$G$47,15)</f>
-        <v/>
-      </c>
-      <c r="C24">
-        <f>COUNTIFS(Trades!$G$2:$G$47,15,Trades!$P$2:$P$47,"Closed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="B25" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,15)</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>COUNTIFS(Trades!$G$2:$G$50,15,Trades!$P$2:$P$50,"Closed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>By Conviction Tier</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>P&amp;L $</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>Win rate</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$Q$2:$Q$47,A29&amp;" *")</f>
-        <v/>
-      </c>
-      <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$47,A29&amp;" *",Trades!$P$2:$P$47,"Closed")</f>
-        <v/>
-      </c>
-      <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$47,A29&amp;" *",Trades!$N$2:$N$47,"&gt;0")/C29)</f>
-        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B30" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$Q$2:$Q$47,A30&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$Q$2:$Q$50,A30&amp;" *")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Trades!$Q$2:$Q$47,A30&amp;" *",Trades!$P$2:$P$47,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$50,A30&amp;" *",Trades!$P$2:$P$50,"Closed")</f>
         <v/>
       </c>
       <c r="D30" s="13">
-        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$47,A30&amp;" *",Trades!$N$2:$N$47,"&gt;0")/C30)</f>
+        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$50,A30&amp;" *",Trades!$N$2:$N$50,"&gt;0")/C30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="B31" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$Q$2:$Q$50,A31&amp;" *")</f>
+        <v/>
+      </c>
+      <c r="C31">
+        <f>COUNTIFS(Trades!$Q$2:$Q$50,A31&amp;" *",Trades!$P$2:$P$50,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D31" s="13">
+        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$50,A31&amp;" *",Trades!$N$2:$N$50,"&gt;0")/C31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="B31" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$47,Trades!$Q$2:$Q$47,A31&amp;" *")</f>
-        <v/>
-      </c>
-      <c r="C31">
-        <f>COUNTIFS(Trades!$Q$2:$Q$47,A31&amp;" *",Trades!$P$2:$P$47,"Closed")</f>
-        <v/>
-      </c>
-      <c r="D31" s="13">
-        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$47,A31&amp;" *",Trades!$N$2:$N$47,"&gt;0")/C31)</f>
+      <c r="B32" s="11">
+        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$Q$2:$Q$50,A32&amp;" *")</f>
+        <v/>
+      </c>
+      <c r="C32">
+        <f>COUNTIFS(Trades!$Q$2:$Q$50,A32&amp;" *",Trades!$P$2:$P$50,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D32" s="13">
+        <f>IF(C32=0,0,COUNTIFS(Trades!$Q$2:$Q$50,A32&amp;" *",Trades!$N$2:$N$50,"&gt;0")/C32)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
timeout on stale orders
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$13</f>
+              <f>'Daily'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$13</f>
+              <f>'Daily'!$B$2:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$13</f>
+              <f>'Daily'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$13</f>
+              <f>'Daily'!$C$2:$C$14</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-14 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-07-15 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$50)</f>
+        <f>SUM(Trades!$N$2:$N$51)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$50,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$51,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$50,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$51,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$50,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$50,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$51,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$51,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$50,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$50,"&gt;0")/SUMIF(Trades!$N$2:$N$50,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$51,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$51,"&gt;0")/SUMIF(Trades!$N$2:$N$51,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$13)</f>
+        <f>MAX(Daily!$B$2:$B$14)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$13)</f>
+        <f>MIN(Daily!$B$2:$B$14)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$50)</f>
+        <f>SUM(Trades!$R$2:$R$51)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4418,6 +4418,76 @@
         <v>20.89</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="9" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>XSP</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>07-15 13:47</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>07-15 13:49</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="H51" s="10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I51" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J51" s="10" t="n">
+        <v>31.82</v>
+      </c>
+      <c r="K51" s="10" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="L51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="6" t="n">
+        <v>-0.2857</v>
+      </c>
+      <c r="N51" s="4" t="n">
+        <v>-80</v>
+      </c>
+      <c r="O51" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P51" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q51" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 2/5 | ADX✓ slope✓ agree✗ early✗ tape✗(20x)</t>
+        </is>
+      </c>
+      <c r="R51" s="4" t="n">
+        <v>63.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4429,7 +4499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4479,7 +4549,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -4487,11 +4557,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -4506,7 +4576,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -4514,11 +4584,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -4533,7 +4603,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -4541,11 +4611,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -4560,7 +4630,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -4568,11 +4638,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -4587,7 +4657,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -4595,11 +4665,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -4614,7 +4684,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -4622,11 +4692,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -4641,7 +4711,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -4649,11 +4719,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -4668,7 +4738,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -4676,11 +4746,11 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
@@ -4695,7 +4765,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -4703,11 +4773,11 @@
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F10">
@@ -4722,7 +4792,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-10")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-10")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -4730,11 +4800,11 @@
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-10")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-10")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-10")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-10")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F11">
@@ -4749,7 +4819,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-13")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-13")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C12" s="11">
@@ -4757,11 +4827,11 @@
         <v/>
       </c>
       <c r="D12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-13")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-13")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-13")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-13")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F12">
@@ -4776,7 +4846,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-14")*Trades!$N$2:$N$50)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-14")*Trades!$N$2:$N$51)</f>
         <v/>
       </c>
       <c r="C13" s="11">
@@ -4784,15 +4854,42 @@
         <v/>
       </c>
       <c r="D13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-14")*(Trades!$P$2:$P$50="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-14")*(Trades!$P$2:$P$51="Closed")*1)</f>
         <v/>
       </c>
       <c r="E13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$50,"yyyy-mm-dd")="2026-07-14")*(Trades!$N$2:$N$50&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-14")*(Trades!$N$2:$N$51&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F13">
         <f>D13-E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07/15</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-15")*Trades!$N$2:$N$51)</f>
+        <v/>
+      </c>
+      <c r="C14" s="11">
+        <f>SUM($B$2:B14)</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-15")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-15")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>D14-E14</f>
         <v/>
       </c>
     </row>
@@ -4852,15 +4949,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$50,A3,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$51,A3,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$50,A3,Trades!$N$2:$N$50,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$51,A3,Trades!$N$2:$N$51,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -4871,15 +4968,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A4)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS(Trades!$B$2:$B$50,A4,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$51,A4,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$50,A4,Trades!$N$2:$N$50,"&gt;0")/C4)</f>
+        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$51,A4,Trades!$N$2:$N$51,"&gt;0")/C4)</f>
         <v/>
       </c>
     </row>
@@ -4890,15 +4987,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A5)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS(Trades!$B$2:$B$50,A5,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$51,A5,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$50,A5,Trades!$N$2:$N$50,"&gt;0")/C5)</f>
+        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$51,A5,Trades!$N$2:$N$51,"&gt;0")/C5)</f>
         <v/>
       </c>
     </row>
@@ -4909,15 +5006,15 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$B$2:$B$50,A6)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A6)</f>
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIFS(Trades!$B$2:$B$50,A6,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$51,A6,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>IF(C6=0,0,COUNTIFS(Trades!$B$2:$B$50,A6,Trades!$N$2:$N$50,"&gt;0")/C6)</f>
+        <f>IF(C6=0,0,COUNTIFS(Trades!$B$2:$B$51,A6,Trades!$N$2:$N$51,"&gt;0")/C6)</f>
         <v/>
       </c>
     </row>
@@ -4957,11 +5054,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$50,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$51,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -4976,11 +5073,11 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIF(Trades!$O$2:$O$50,A12)</f>
+        <f>COUNTIF(Trades!$O$2:$O$51,A12)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -4995,11 +5092,11 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIF(Trades!$O$2:$O$50,A13)</f>
+        <f>COUNTIF(Trades!$O$2:$O$51,A13)</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -5014,11 +5111,11 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$O$2:$O$50,A14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A14)</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIF(Trades!$O$2:$O$50,A14)</f>
+        <f>COUNTIF(Trades!$O$2:$O$51,A14)</f>
         <v/>
       </c>
       <c r="D14" s="11">
@@ -5057,11 +5154,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,9)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$50,9,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,9,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5072,11 +5169,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,10)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$50,10,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,10,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5087,11 +5184,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,11)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$50,11,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,11,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5102,11 +5199,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,12)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$50,12,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,12,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5117,11 +5214,11 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,13)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Trades!$G$2:$G$50,13,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,13,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5132,11 +5229,11 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,14)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Trades!$G$2:$G$50,14,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,14,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5147,11 +5244,11 @@
         </is>
       </c>
       <c r="B25" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$G$2:$G$50,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,15)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Trades!$G$2:$G$50,15,Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$51,15,Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5191,15 +5288,15 @@
         </is>
       </c>
       <c r="B30" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$Q$2:$Q$50,A30&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$Q$2:$Q$51,A30&amp;" *")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Trades!$Q$2:$Q$50,A30&amp;" *",Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$51,A30&amp;" *",Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D30" s="13">
-        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$50,A30&amp;" *",Trades!$N$2:$N$50,"&gt;0")/C30)</f>
+        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$51,A30&amp;" *",Trades!$N$2:$N$51,"&gt;0")/C30)</f>
         <v/>
       </c>
     </row>
@@ -5210,15 +5307,15 @@
         </is>
       </c>
       <c r="B31" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$Q$2:$Q$50,A31&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$Q$2:$Q$51,A31&amp;" *")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS(Trades!$Q$2:$Q$50,A31&amp;" *",Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$51,A31&amp;" *",Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D31" s="13">
-        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$50,A31&amp;" *",Trades!$N$2:$N$50,"&gt;0")/C31)</f>
+        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$51,A31&amp;" *",Trades!$N$2:$N$51,"&gt;0")/C31)</f>
         <v/>
       </c>
     </row>
@@ -5229,15 +5326,15 @@
         </is>
       </c>
       <c r="B32" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$50,Trades!$Q$2:$Q$50,A32&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$Q$2:$Q$51,A32&amp;" *")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS(Trades!$Q$2:$Q$50,A32&amp;" *",Trades!$P$2:$P$50,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$51,A32&amp;" *",Trades!$P$2:$P$51,"Closed")</f>
         <v/>
       </c>
       <c r="D32" s="13">
-        <f>IF(C32=0,0,COUNTIFS(Trades!$Q$2:$Q$50,A32&amp;" *",Trades!$N$2:$N$50,"&gt;0")/C32)</f>
+        <f>IF(C32=0,0,COUNTIFS(Trades!$Q$2:$Q$51,A32&amp;" *",Trades!$N$2:$N$51,"&gt;0")/C32)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
latest data from runs
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$14</f>
+              <f>'Daily'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$14</f>
+              <f>'Daily'!$B$2:$B$15</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$14</f>
+              <f>'Daily'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$14</f>
+              <f>'Daily'!$C$2:$C$15</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-15 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-07-17 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$51)</f>
+        <f>SUM(Trades!$N$2:$N$54)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$51,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$54,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$51,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$54,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$51,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$51,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$54,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$54,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$51,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$51,"&gt;0")/SUMIF(Trades!$N$2:$N$51,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$54,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$54,"&gt;0")/SUMIF(Trades!$N$2:$N$54,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$14)</f>
+        <f>MAX(Daily!$B$2:$B$15)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$14)</f>
+        <f>MIN(Daily!$B$2:$B$15)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$51)</f>
+        <f>SUM(Trades!$R$2:$R$54)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R51"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4488,6 +4488,164 @@
         <v>63.62</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="9" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>XSP</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>07-15 17:42</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="H52" s="10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I52" s="10" t="n"/>
+      <c r="J52" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K52" s="10" t="n"/>
+      <c r="L52" s="6" t="n"/>
+      <c r="M52" s="6" t="n"/>
+      <c r="N52" s="4" t="n"/>
+      <c r="O52" s="10" t="inlineStr"/>
+      <c r="P52" s="10" t="inlineStr">
+        <is>
+          <t>Orphaned/manual</t>
+        </is>
+      </c>
+      <c r="Q52" s="10" t="inlineStr"/>
+      <c r="R52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>XSP</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>07-15 17:42</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr"/>
+      <c r="F53" s="10" t="n"/>
+      <c r="G53" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="H53" s="10" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="I53" s="10" t="n"/>
+      <c r="J53" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K53" s="10" t="n"/>
+      <c r="L53" s="6" t="n"/>
+      <c r="M53" s="6" t="n"/>
+      <c r="N53" s="4" t="n"/>
+      <c r="O53" s="10" t="inlineStr"/>
+      <c r="P53" s="10" t="inlineStr">
+        <is>
+          <t>Orphaned/manual</t>
+        </is>
+      </c>
+      <c r="Q53" s="10" t="inlineStr"/>
+      <c r="R53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>XSP</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>07-16 10:31</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>07-16 10:56</t>
+        </is>
+      </c>
+      <c r="F54" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="G54" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H54" s="10" t="n">
+        <v>0.468333</v>
+      </c>
+      <c r="I54" s="10" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J54" s="10" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="K54" s="10" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="L54" s="6" t="n">
+        <v>0.0356</v>
+      </c>
+      <c r="M54" s="6" t="n">
+        <v>-0.274</v>
+      </c>
+      <c r="N54" s="4" t="n">
+        <v>-77</v>
+      </c>
+      <c r="O54" s="10" t="inlineStr">
+        <is>
+          <t>Invalidation</t>
+        </is>
+      </c>
+      <c r="P54" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q54" s="10" t="inlineStr">
+        <is>
+          <t>MEDIUM 2/5 | ADX✓ slope✗ agree✗ early✓ tape✗(5x)</t>
+        </is>
+      </c>
+      <c r="R54" s="4" t="n">
+        <v>20.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4499,7 +4657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4549,7 +4707,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-05-05")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -4557,11 +4715,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-05-05")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-05-05")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -4576,7 +4734,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-05-15")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -4584,11 +4742,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-05-15")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-05-15")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -4603,7 +4761,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-06-29")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -4611,11 +4769,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-06-29")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-06-29")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -4630,7 +4788,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-06-30")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -4638,11 +4796,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-06-30")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-06-30")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -4657,7 +4815,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-01")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -4665,11 +4823,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-01")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-01")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -4684,7 +4842,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-06")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -4692,11 +4850,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-06")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-06")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -4711,7 +4869,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-07")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -4719,11 +4877,11 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-07")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-07")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
@@ -4738,7 +4896,7 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-08")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C9" s="11">
@@ -4746,11 +4904,11 @@
         <v/>
       </c>
       <c r="D9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-08")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E9">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-08")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F9">
@@ -4765,7 +4923,7 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-09")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C10" s="11">
@@ -4773,11 +4931,11 @@
         <v/>
       </c>
       <c r="D10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-09")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E10">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-09")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F10">
@@ -4792,7 +4950,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-10")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-10")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C11" s="11">
@@ -4800,11 +4958,11 @@
         <v/>
       </c>
       <c r="D11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-10")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-10")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-10")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-10")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F11">
@@ -4819,7 +4977,7 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-13")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-13")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C12" s="11">
@@ -4827,11 +4985,11 @@
         <v/>
       </c>
       <c r="D12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-13")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-13")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E12">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-13")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-13")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F12">
@@ -4846,7 +5004,7 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-14")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-14")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C13" s="11">
@@ -4854,11 +5012,11 @@
         <v/>
       </c>
       <c r="D13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-14")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-14")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E13">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-14")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-14")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F13">
@@ -4873,7 +5031,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-15")*Trades!$N$2:$N$51)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-15")*Trades!$N$2:$N$54)</f>
         <v/>
       </c>
       <c r="C14" s="11">
@@ -4881,15 +5039,42 @@
         <v/>
       </c>
       <c r="D14">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-15")*(Trades!$P$2:$P$51="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-15")*(Trades!$P$2:$P$54="Closed")*1)</f>
         <v/>
       </c>
       <c r="E14">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$51,"yyyy-mm-dd")="2026-07-15")*(Trades!$N$2:$N$51&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-15")*(Trades!$N$2:$N$54&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F14">
         <f>D14-E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07/16</t>
+        </is>
+      </c>
+      <c r="B15" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-16")*Trades!$N$2:$N$54)</f>
+        <v/>
+      </c>
+      <c r="C15" s="11">
+        <f>SUM($B$2:B15)</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-16")*(Trades!$P$2:$P$54="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$54,"yyyy-mm-dd")="2026-07-16")*(Trades!$N$2:$N$54&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>D15-E15</f>
         <v/>
       </c>
     </row>
@@ -4949,15 +5134,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$B$2:$B$54,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$51,A3,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$54,A3,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$51,A3,Trades!$N$2:$N$51,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$54,A3,Trades!$N$2:$N$54,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -4968,15 +5153,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A4)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$B$2:$B$54,A4)</f>
         <v/>
       </c>
       <c r="C4">
-        <f>COUNTIFS(Trades!$B$2:$B$51,A4,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$54,A4,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$51,A4,Trades!$N$2:$N$51,"&gt;0")/C4)</f>
+        <f>IF(C4=0,0,COUNTIFS(Trades!$B$2:$B$54,A4,Trades!$N$2:$N$54,"&gt;0")/C4)</f>
         <v/>
       </c>
     </row>
@@ -4987,15 +5172,15 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A5)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$B$2:$B$54,A5)</f>
         <v/>
       </c>
       <c r="C5">
-        <f>COUNTIFS(Trades!$B$2:$B$51,A5,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$54,A5,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$51,A5,Trades!$N$2:$N$51,"&gt;0")/C5)</f>
+        <f>IF(C5=0,0,COUNTIFS(Trades!$B$2:$B$54,A5,Trades!$N$2:$N$54,"&gt;0")/C5)</f>
         <v/>
       </c>
     </row>
@@ -5006,15 +5191,15 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$B$2:$B$51,A6)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$B$2:$B$54,A6)</f>
         <v/>
       </c>
       <c r="C6">
-        <f>COUNTIFS(Trades!$B$2:$B$51,A6,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$54,A6,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>IF(C6=0,0,COUNTIFS(Trades!$B$2:$B$51,A6,Trades!$N$2:$N$51,"&gt;0")/C6)</f>
+        <f>IF(C6=0,0,COUNTIFS(Trades!$B$2:$B$54,A6,Trades!$N$2:$N$54,"&gt;0")/C6)</f>
         <v/>
       </c>
     </row>
@@ -5054,11 +5239,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$O$2:$O$54,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$51,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$54,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -5073,11 +5258,11 @@
         </is>
       </c>
       <c r="B12" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$O$2:$O$54,A12)</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIF(Trades!$O$2:$O$51,A12)</f>
+        <f>COUNTIF(Trades!$O$2:$O$54,A12)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -5092,11 +5277,11 @@
         </is>
       </c>
       <c r="B13" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$O$2:$O$54,A13)</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIF(Trades!$O$2:$O$51,A13)</f>
+        <f>COUNTIF(Trades!$O$2:$O$54,A13)</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -5111,11 +5296,11 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$O$2:$O$51,A14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$O$2:$O$54,A14)</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIF(Trades!$O$2:$O$51,A14)</f>
+        <f>COUNTIF(Trades!$O$2:$O$54,A14)</f>
         <v/>
       </c>
       <c r="D14" s="11">
@@ -5154,11 +5339,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,9)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$51,9,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,9,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5169,11 +5354,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,10)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$51,10,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,10,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5184,11 +5369,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,11)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$51,11,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,11,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5199,11 +5384,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,12)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$51,12,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,12,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5214,11 +5399,11 @@
         </is>
       </c>
       <c r="B23" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,13)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Trades!$G$2:$G$51,13,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,13,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5229,11 +5414,11 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,14)</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Trades!$G$2:$G$51,14,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,14,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5244,11 +5429,11 @@
         </is>
       </c>
       <c r="B25" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$G$2:$G$51,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$G$2:$G$54,15)</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Trades!$G$2:$G$51,15,Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$54,15,Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -5288,15 +5473,15 @@
         </is>
       </c>
       <c r="B30" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$Q$2:$Q$51,A30&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$Q$2:$Q$54,A30&amp;" *")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Trades!$Q$2:$Q$51,A30&amp;" *",Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$54,A30&amp;" *",Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D30" s="13">
-        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$51,A30&amp;" *",Trades!$N$2:$N$51,"&gt;0")/C30)</f>
+        <f>IF(C30=0,0,COUNTIFS(Trades!$Q$2:$Q$54,A30&amp;" *",Trades!$N$2:$N$54,"&gt;0")/C30)</f>
         <v/>
       </c>
     </row>
@@ -5307,15 +5492,15 @@
         </is>
       </c>
       <c r="B31" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$Q$2:$Q$51,A31&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$Q$2:$Q$54,A31&amp;" *")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS(Trades!$Q$2:$Q$51,A31&amp;" *",Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$54,A31&amp;" *",Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D31" s="13">
-        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$51,A31&amp;" *",Trades!$N$2:$N$51,"&gt;0")/C31)</f>
+        <f>IF(C31=0,0,COUNTIFS(Trades!$Q$2:$Q$54,A31&amp;" *",Trades!$N$2:$N$54,"&gt;0")/C31)</f>
         <v/>
       </c>
     </row>
@@ -5326,15 +5511,15 @@
         </is>
       </c>
       <c r="B32" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$51,Trades!$Q$2:$Q$51,A32&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$54,Trades!$Q$2:$Q$54,A32&amp;" *")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS(Trades!$Q$2:$Q$51,A32&amp;" *",Trades!$P$2:$P$51,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$54,A32&amp;" *",Trades!$P$2:$P$54,"Closed")</f>
         <v/>
       </c>
       <c r="D32" s="13">
-        <f>IF(C32=0,0,COUNTIFS(Trades!$Q$2:$Q$51,A32&amp;" *",Trades!$N$2:$N$51,"&gt;0")/C32)</f>
+        <f>IF(C32=0,0,COUNTIFS(Trades!$Q$2:$Q$54,A32&amp;" *",Trades!$N$2:$N$54,"&gt;0")/C32)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
adding max adverse pct and gex data
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$4</f>
+              <f>'Daily'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$4</f>
+              <f>'Daily'!$B$2:$B$5</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$4</f>
+              <f>'Daily'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$4</f>
+              <f>'Daily'!$C$2:$C$5</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-19 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-08-20 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$4)</f>
+        <f>SUM(Trades!$N$2:$N$5)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$4,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$5,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$4,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$5,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$4,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$4,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$5,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$5,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$4,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$4,"&gt;0")/SUMIF(Trades!$N$2:$N$4,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$5,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$5,"&gt;0")/SUMIF(Trades!$N$2:$N$5,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$4)</f>
+        <f>MAX(Daily!$B$2:$B$5)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$4)</f>
+        <f>MIN(Daily!$B$2:$B$5)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$4)</f>
+        <f>SUM(Trades!$R$2:$R$5)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1538,6 +1538,68 @@
         <v>3.26</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>08-20 10:17</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>08-20 14:12</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>235</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="6" t="n">
+        <v>0.7929999999999999</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>0.6328</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>810</v>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr"/>
+      <c r="R5" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1549,7 +1611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1599,7 +1661,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$4)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$5)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -1607,11 +1669,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$4="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$5="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$4&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$5&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -1626,7 +1688,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$4)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$5)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -1634,11 +1696,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$4="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$5="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$4&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$5&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -1653,7 +1715,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$4)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$5)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -1661,15 +1723,42 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$4="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$5="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$4,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$4&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$5&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
         <f>D4-E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>08/20</t>
+        </is>
+      </c>
+      <c r="B5" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="11">
+        <f>SUM($B$2:B5)</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$5="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$5,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$5&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>D5-E5</f>
         <v/>
       </c>
     </row>
@@ -1729,15 +1818,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$B$2:$B$4,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$B$2:$B$5,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$4,A3,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$5,A3,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$4,A3,Trades!$N$2:$N$4,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$5,A3,Trades!$N$2:$N$5,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -1777,11 +1866,11 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$O$2:$O$4,A8)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$O$2:$O$5,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIF(Trades!$O$2:$O$4,A8)</f>
+        <f>COUNTIF(Trades!$O$2:$O$5,A8)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -1796,11 +1885,11 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$O$2:$O$4,A9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$O$2:$O$5,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIF(Trades!$O$2:$O$4,A9)</f>
+        <f>COUNTIF(Trades!$O$2:$O$5,A9)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -1815,11 +1904,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$O$2:$O$4,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$O$2:$O$5,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$4,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$5,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -1834,11 +1923,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$O$2:$O$4,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$O$2:$O$5,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$4,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$5,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -1877,11 +1966,11 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,9)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Trades!$G$2:$G$4,9,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,9,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1892,11 +1981,11 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,10)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Trades!$G$2:$G$4,10,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,10,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1907,11 +1996,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,11)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$4,11,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,11,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1922,11 +2011,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,12)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$4,12,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,12,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1937,11 +2026,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,13)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$4,13,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,13,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1952,11 +2041,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,14)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$4,14,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,14,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1967,11 +2056,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$G$2:$G$4,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$G$2:$G$5,15)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$4,15,Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$5,15,Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2011,15 +2100,15 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$Q$2:$Q$4,A27&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$Q$2:$Q$5,A27&amp;" *")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Trades!$Q$2:$Q$4,A27&amp;" *",Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$5,A27&amp;" *",Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
       <c r="D27" s="13">
-        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$4,A27&amp;" *",Trades!$N$2:$N$4,"&gt;0")/C27)</f>
+        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$5,A27&amp;" *",Trades!$N$2:$N$5,"&gt;0")/C27)</f>
         <v/>
       </c>
     </row>
@@ -2030,15 +2119,15 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$Q$2:$Q$4,A28&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$Q$2:$Q$5,A28&amp;" *")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Trades!$Q$2:$Q$4,A28&amp;" *",Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$5,A28&amp;" *",Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
       <c r="D28" s="13">
-        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$4,A28&amp;" *",Trades!$N$2:$N$4,"&gt;0")/C28)</f>
+        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$5,A28&amp;" *",Trades!$N$2:$N$5,"&gt;0")/C28)</f>
         <v/>
       </c>
     </row>
@@ -2049,15 +2138,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$4,Trades!$Q$2:$Q$4,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$5,Trades!$Q$2:$Q$5,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$4,A29&amp;" *",Trades!$P$2:$P$4,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$5,A29&amp;" *",Trades!$P$2:$P$5,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$4,A29&amp;" *",Trades!$N$2:$N$4,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$5,A29&amp;" *",Trades!$N$2:$N$5,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
gex data and trailing tiers
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -217,12 +217,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$8</f>
+              <f>'Daily'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$B$2:$B$8</f>
+              <f>'Daily'!$B$2:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -304,12 +304,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Daily'!$A$2:$A$8</f>
+              <f>'Daily'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Daily'!$C$2:$C$8</f>
+              <f>'Daily'!$C$2:$C$9</f>
             </numRef>
           </val>
         </ser>
@@ -1113,7 +1113,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-25 15:00 — refresh: python scripts/build_dashboard.py</t>
+          <t>Generated 2026-08-27 15:00 — refresh: python scripts/build_dashboard.py</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUM(Trades!$N$2:$N$10)</f>
+        <f>SUM(Trades!$N$2:$N$12)</f>
         <v/>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIF(Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF(Trades!$N$2:$N$10,"&gt;0")/B5</f>
+        <f>COUNTIF(Trades!$N$2:$N$12,"&gt;0")/B5</f>
         <v/>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>AVERAGEIF(Trades!$N$2:$N$10,"&gt;0")</f>
+        <f>AVERAGEIF(Trades!$N$2:$N$12,"&gt;0")</f>
         <v/>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>IF(COUNTIF(Trades!$N$2:$N$10,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$10,"&lt;0"))</f>
+        <f>IF(COUNTIF(Trades!$N$2:$N$12,"&lt;0")=0,0,AVERAGEIF(Trades!$N$2:$N$12,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>IF(SUMIF(Trades!$N$2:$N$10,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$10,"&gt;0")/SUMIF(Trades!$N$2:$N$10,"&lt;0"))</f>
+        <f>IF(SUMIF(Trades!$N$2:$N$12,"&lt;0")=0,0,-SUMIF(Trades!$N$2:$N$12,"&gt;0")/SUMIF(Trades!$N$2:$N$12,"&lt;0"))</f>
         <v/>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>MAX(Daily!$B$2:$B$8)</f>
+        <f>MAX(Daily!$B$2:$B$9)</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="B11" s="4">
-        <f>MIN(Daily!$B$2:$B$8)</f>
+        <f>MIN(Daily!$B$2:$B$9)</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="B12" s="4">
-        <f>SUM(Trades!$R$2:$R$10)</f>
+        <f>SUM(Trades!$R$2:$R$12)</f>
         <v/>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1880,6 +1880,130 @@
         <v>3.26</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>08-27 09:33</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>08-27 09:42</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="J11" s="10" t="n"/>
+      <c r="K11" s="10" t="n"/>
+      <c r="L11" s="6" t="n">
+        <v>0.3611</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.2778</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>400</v>
+      </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr"/>
+      <c r="R11" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>08-27 09:55</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>08-27 11:03</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>69</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="J12" s="10" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="6" t="n">
+        <v>0.4385</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>0.3385</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>440</v>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P12" s="10" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr"/>
+      <c r="R12" s="4" t="n">
+        <v>3.26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1891,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1941,7 +2065,7 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-17")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C2" s="11">
@@ -1949,11 +2073,11 @@
         <v/>
       </c>
       <c r="D2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-17")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E2">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-17")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F2">
@@ -1968,7 +2092,7 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-18")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C3" s="11">
@@ -1976,11 +2100,11 @@
         <v/>
       </c>
       <c r="D3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-18")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E3">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-18")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F3">
@@ -1995,7 +2119,7 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-19")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -2003,11 +2127,11 @@
         <v/>
       </c>
       <c r="D4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-19")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E4">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-19")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F4">
@@ -2022,7 +2146,7 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-20")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -2030,11 +2154,11 @@
         <v/>
       </c>
       <c r="D5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-20")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-20")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F5">
@@ -2049,7 +2173,7 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-21")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -2057,11 +2181,11 @@
         <v/>
       </c>
       <c r="D6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-21")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E6">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-21")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F6">
@@ -2076,7 +2200,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-24")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C7" s="11">
@@ -2084,11 +2208,11 @@
         <v/>
       </c>
       <c r="D7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-24")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E7">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-24")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F7">
@@ -2103,7 +2227,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$10)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-25")*Trades!$N$2:$N$12)</f>
         <v/>
       </c>
       <c r="C8" s="11">
@@ -2111,15 +2235,42 @@
         <v/>
       </c>
       <c r="D8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$10="Closed")*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-25")*(Trades!$P$2:$P$12="Closed")*1)</f>
         <v/>
       </c>
       <c r="E8">
-        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$10,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$10&gt;0)*1)</f>
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-25")*(Trades!$N$2:$N$12&gt;0)*1)</f>
         <v/>
       </c>
       <c r="F8">
         <f>D8-E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>08/27</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-27")*Trades!$N$2:$N$12)</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>SUM($B$2:B9)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-27")*(Trades!$P$2:$P$12="Closed")*1)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SUMPRODUCT((TEXT(Trades!$A$2:$A$12,"yyyy-mm-dd")="2026-08-27")*(Trades!$N$2:$N$12&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>D9-E9</f>
         <v/>
       </c>
     </row>
@@ -2179,15 +2330,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$B$2:$B$10,A3)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$B$2:$B$12,A3)</f>
         <v/>
       </c>
       <c r="C3">
-        <f>COUNTIFS(Trades!$B$2:$B$10,A3,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$B$2:$B$12,A3,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$10,A3,Trades!$N$2:$N$10,"&gt;0")/C3)</f>
+        <f>IF(C3=0,0,COUNTIFS(Trades!$B$2:$B$12,A3,Trades!$N$2:$N$12,"&gt;0")/C3)</f>
         <v/>
       </c>
     </row>
@@ -2227,11 +2378,11 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$O$2:$O$10,A8)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$O$2:$O$12,A8)</f>
         <v/>
       </c>
       <c r="C8">
-        <f>COUNTIF(Trades!$O$2:$O$10,A8)</f>
+        <f>COUNTIF(Trades!$O$2:$O$12,A8)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -2246,11 +2397,11 @@
         </is>
       </c>
       <c r="B9" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$O$2:$O$10,A9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$O$2:$O$12,A9)</f>
         <v/>
       </c>
       <c r="C9">
-        <f>COUNTIF(Trades!$O$2:$O$10,A9)</f>
+        <f>COUNTIF(Trades!$O$2:$O$12,A9)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -2265,11 +2416,11 @@
         </is>
       </c>
       <c r="B10" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$O$2:$O$10,A10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$O$2:$O$12,A10)</f>
         <v/>
       </c>
       <c r="C10">
-        <f>COUNTIF(Trades!$O$2:$O$10,A10)</f>
+        <f>COUNTIF(Trades!$O$2:$O$12,A10)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -2284,11 +2435,11 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$O$2:$O$10,A11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$O$2:$O$12,A11)</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIF(Trades!$O$2:$O$10,A11)</f>
+        <f>COUNTIF(Trades!$O$2:$O$12,A11)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -2327,11 +2478,11 @@
         </is>
       </c>
       <c r="B16" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,9)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,9)</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Trades!$G$2:$G$10,9,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,9,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2342,11 +2493,11 @@
         </is>
       </c>
       <c r="B17" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,10)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,10)</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Trades!$G$2:$G$10,10,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,10,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2357,11 +2508,11 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,11)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,11)</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Trades!$G$2:$G$10,11,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,11,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2372,11 +2523,11 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,12)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,12)</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Trades!$G$2:$G$10,12,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,12,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2387,11 +2538,11 @@
         </is>
       </c>
       <c r="B20" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,13)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,13)</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Trades!$G$2:$G$10,13,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,13,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2402,11 +2553,11 @@
         </is>
       </c>
       <c r="B21" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,14)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,14)</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Trades!$G$2:$G$10,14,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,14,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2417,11 +2568,11 @@
         </is>
       </c>
       <c r="B22" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$G$2:$G$10,15)</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$G$2:$G$12,15)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Trades!$G$2:$G$10,15,Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$G$2:$G$12,15,Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
     </row>
@@ -2461,15 +2612,15 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$Q$2:$Q$10,A27&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$Q$2:$Q$12,A27&amp;" *")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Trades!$Q$2:$Q$10,A27&amp;" *",Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$12,A27&amp;" *",Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
       <c r="D27" s="13">
-        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$10,A27&amp;" *",Trades!$N$2:$N$10,"&gt;0")/C27)</f>
+        <f>IF(C27=0,0,COUNTIFS(Trades!$Q$2:$Q$12,A27&amp;" *",Trades!$N$2:$N$12,"&gt;0")/C27)</f>
         <v/>
       </c>
     </row>
@@ -2480,15 +2631,15 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$Q$2:$Q$10,A28&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$Q$2:$Q$12,A28&amp;" *")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Trades!$Q$2:$Q$10,A28&amp;" *",Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$12,A28&amp;" *",Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
       <c r="D28" s="13">
-        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$10,A28&amp;" *",Trades!$N$2:$N$10,"&gt;0")/C28)</f>
+        <f>IF(C28=0,0,COUNTIFS(Trades!$Q$2:$Q$12,A28&amp;" *",Trades!$N$2:$N$12,"&gt;0")/C28)</f>
         <v/>
       </c>
     </row>
@@ -2499,15 +2650,15 @@
         </is>
       </c>
       <c r="B29" s="11">
-        <f>SUMIFS(Trades!$N$2:$N$10,Trades!$Q$2:$Q$10,A29&amp;" *")</f>
+        <f>SUMIFS(Trades!$N$2:$N$12,Trades!$Q$2:$Q$12,A29&amp;" *")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Trades!$Q$2:$Q$10,A29&amp;" *",Trades!$P$2:$P$10,"Closed")</f>
+        <f>COUNTIFS(Trades!$Q$2:$Q$12,A29&amp;" *",Trades!$P$2:$P$12,"Closed")</f>
         <v/>
       </c>
       <c r="D29" s="13">
-        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$10,A29&amp;" *",Trades!$N$2:$N$10,"&gt;0")/C29)</f>
+        <f>IF(C29=0,0,COUNTIFS(Trades!$Q$2:$Q$12,A29&amp;" *",Trades!$N$2:$N$12,"&gt;0")/C29)</f>
         <v/>
       </c>
     </row>

</xml_diff>